<commit_message>
feat: improved liquibase handling
</commit_message>
<xml_diff>
--- a/docs/liquibase/liquibase.xlsx
+++ b/docs/liquibase/liquibase.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Process Step ID</t>
   </si>
@@ -34,13 +34,13 @@
     <t>Owner / Function</t>
   </si>
   <si>
-    <t>C:\Users\U00001\source\repos\etl-madness\CodeFlow\examples\liquibase\01_core_schema.xml:1:8</t>
+    <t>examples\liquibase\changeset\core_changeset.1.xml:1:8</t>
   </si>
   <si>
     <t>Create customers table</t>
   </si>
   <si>
-    <t>C:\Users\U00001\source\repos\etl-madness\CodeFlow\examples\liquibase\01_core_schema.xml:2:30</t>
+    <t>examples\liquibase\changeset\core_changeset.1.xml:2:30</t>
   </si>
   <si>
     <t>executes next</t>
@@ -49,25 +49,76 @@
     <t>TableOperation</t>
   </si>
   <si>
-    <t>Liquibase (01_core_schema)</t>
+    <t>Liquibase (core_changeset.1)</t>
   </si>
   <si>
     <t>Create merchants table</t>
   </si>
   <si>
-    <t>C:\Users\U00001\source\repos\etl-madness\CodeFlow\examples\liquibase\01_core_schema.xml:3:49</t>
+    <t>examples\liquibase\changeset\core_changeset.1.xml:3:49</t>
   </si>
   <si>
     <t>Create index idx_customers_email on customers; Tag database milestone: v1.0-baseline</t>
   </si>
   <si>
+    <t>examples\liquibase\changeset\customer_changeset.1.xml:dbbo_usp_GetCustomer.1:10</t>
+  </si>
+  <si>
+    <t>Milestone</t>
+  </si>
+  <si>
+    <t>Execute &lt;sqlFile&gt;: dbo_usp_GetCustomer.1.sql</t>
+  </si>
+  <si>
+    <t>examples\liquibase\changeset\sql_changeset.1.sql:orders-v1:3, examples\liquibase\ddl\dbo_usp_GetCustomer.1.sql:stmt:1</t>
+  </si>
+  <si>
+    <t>executes next, calls &lt;sqlFile&gt;</t>
+  </si>
+  <si>
+    <t>StoredProcedure</t>
+  </si>
+  <si>
+    <t>Liquibase (customer_changeset.1)</t>
+  </si>
+  <si>
+    <t>examples\liquibase\changeset\sql_changeset.1.sql:orders-v1:3</t>
+  </si>
+  <si>
+    <t>Create orders table with foreign keys to customers and merchants</t>
+  </si>
+  <si>
+    <t>examples\liquibase\changeset\sql_changeset.1.sql:payments-v1:17</t>
+  </si>
+  <si>
+    <t>Liquibase (sql_changeset.1)</t>
+  </si>
+  <si>
+    <t>Create payments table with foreign key to orders</t>
+  </si>
+  <si>
+    <t>examples\liquibase\changeset\sql_changeset.1.sql:views-and-procs:31</t>
+  </si>
+  <si>
+    <t>Create analytics view for merchant billing</t>
+  </si>
+  <si>
+    <t>examples\liquibase\changeset\sql_changeset.1.sql:milestone-v1.1:43</t>
+  </si>
+  <si>
+    <t>DatabaseView</t>
+  </si>
+  <si>
+    <t>Tag database release milestone</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Milestone</t>
-  </si>
-  <si>
-    <t>C:\Users\U00001\source\repos\etl-madness\CodeFlow\examples\liquibase\01_core_schema.xml:table:customers</t>
+    <t>DatabaseQuery</t>
+  </si>
+  <si>
+    <t>examples\liquibase\changeset\core_changeset.1.xml:table:customers</t>
   </si>
   <si>
     <t>Customer profile and authentication records</t>
@@ -76,64 +127,49 @@
     <t>DatabaseTable</t>
   </si>
   <si>
-    <t>C:\Users\U00001\source\repos\etl-madness\CodeFlow\examples\liquibase\01_core_schema.xml:table:merchants</t>
+    <t>examples\liquibase\changeset\core_changeset.1.xml:table:merchants</t>
   </si>
   <si>
     <t>Merchant store entities</t>
   </si>
   <si>
-    <t>C:\Users\U00001\source\repos\etl-madness\CodeFlow\examples\liquibase\02_orders_and_payments.sql:orders-v1:3</t>
-  </si>
-  <si>
-    <t>Create orders table with foreign keys to customers and merchants</t>
-  </si>
-  <si>
-    <t>C:\Users\U00001\source\repos\etl-madness\CodeFlow\examples\liquibase\02_orders_and_payments.sql:payments-v1:17</t>
-  </si>
-  <si>
-    <t>Liquibase (02_orders_and_payments)</t>
-  </si>
-  <si>
-    <t>Create payments table with foreign key to orders</t>
-  </si>
-  <si>
-    <t>C:\Users\U00001\source\repos\etl-madness\CodeFlow\examples\liquibase\02_orders_and_payments.sql:views-and-procs:31</t>
-  </si>
-  <si>
-    <t>Create analytics view for merchant billing</t>
-  </si>
-  <si>
-    <t>C:\Users\U00001\source\repos\etl-madness\CodeFlow\examples\liquibase\02_orders_and_payments.sql:milestone-v1.1:43</t>
-  </si>
-  <si>
-    <t>View</t>
-  </si>
-  <si>
-    <t>Tag database release milestone</t>
-  </si>
-  <si>
-    <t>DatabaseQuery</t>
-  </si>
-  <si>
-    <t>C:\Users\U00001\source\repos\etl-madness\CodeFlow\examples\liquibase\02_orders_and_payments.sql:table:orders</t>
+    <t>examples\liquibase\changeset\sql_changeset.1.sql:table:orders</t>
   </si>
   <si>
     <t>Database Table orders</t>
   </si>
   <si>
-    <t>C:\Users\U00001\source\repos\etl-madness\CodeFlow\examples\liquibase\01_core_schema.xml:table:customers, C:\Users\U00001\source\repos\etl-madness\CodeFlow\examples\liquibase\01_core_schema.xml:table:merchants</t>
+    <t>examples\liquibase\changeset\core_changeset.1.xml:table:customers, examples\liquibase\changeset\core_changeset.1.xml:table:merchants</t>
   </si>
   <si>
     <t>references (fk_orders_customer), references (fk_orders_merchant)</t>
   </si>
   <si>
-    <t>C:\Users\U00001\source\repos\etl-madness\CodeFlow\examples\liquibase\02_orders_and_payments.sql:table:payments</t>
+    <t>examples\liquibase\changeset\sql_changeset.1.sql:table:payments</t>
   </si>
   <si>
     <t>Database Table payments</t>
   </si>
   <si>
     <t>references (fk_payments_order)</t>
+  </si>
+  <si>
+    <t>examples\liquibase\ddl\dbo_usp_GetCustomer.1.sql:stmt:1</t>
+  </si>
+  <si>
+    <t>Stored Procedure Proc: usp_GetCustomer</t>
+  </si>
+  <si>
+    <t>examples\liquibase\ddl\dbo_usp_GetCustomer.1.sql:stmt:1:inner_select:Customer</t>
+  </si>
+  <si>
+    <t>queries</t>
+  </si>
+  <si>
+    <t>SQL Database (dbo_usp_GetCustomer.1)</t>
+  </si>
+  <si>
+    <t>Reads table Customer within stored procedure usp_GetCustomer</t>
   </si>
 </sst>
 </file>
@@ -535,7 +571,7 @@
         <v>15</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>16</v>
@@ -546,53 +582,53 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>9</v>
@@ -606,19 +642,19 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>25</v>
@@ -626,19 +662,19 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>25</v>
@@ -646,62 +682,122 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="F11" s="2" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>